<commit_message>
Adiciona lançamento: maiora (12/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -70,11 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -477,6 +482,31 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>maiora</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>notes de frais hors séjour</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: castelo svevo - repérage (12/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -507,6 +507,31 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>castelo svevo - repérage</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>